<commit_message>
Add live grant shortlist and blockers
<USER ORIGINAL CONVERSATION WITH AGENT>
so search and aply only for oens cna aplya t thtis point nda wiht valeirio
</USER ORIGINAL CONVERSATION WITH AGENT>

Researched live March 2026 opportunities and updated the repo shortlist to distinguish open calls from truly submittable ones.
Marked Eurostars Call 10 as a real but conditional same-week option pending legal and financial eligibility checks for the UK and Spanish SMEs.
Added the EIT Health Innovation Validation Call 2026 as an open next-wave opportunity that fits the project but is not immediate without an additional research or education partner and maturity evidence.
Updated the grant tracker workbook and status file so the repo now reflects the current live landscape: AI Champions ready pending login, Eurostars conditional, EIT Health open but not ready, CARE-03 blocked, EIC already submitted.
</commit_message>
<xml_diff>
--- a/UMBRAMED_GrantApplicationsTracker.xlsx
+++ b/UMBRAMED_GrantApplicationsTracker.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -876,6 +876,162 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Eurostars Call 10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Eurostars-3 Call 10</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>International SME R&amp;D project</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CONDITIONAL - LEGAL CHECKS NEEDED</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Agents AI Ltd</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Eurostars portal / national bodies</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Call 10</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-03-19 14:00 Brussels</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>National funding by country</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Sami + Valerio</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Need immediate SME eligibility/account filings confirmation for Spain and UK</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Only submit if both entities are eligible SMEs and dossier can be assembled immediately</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>GRANT_APPLICATIONS_STATUS.md</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Potentially real, but only with same-week legal/financial confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EIT Health Innovation Validation Call 2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EIT Health Innovation Validation Call 2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Consortium validation grant</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OPEN - NOT READY</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Agents AI Ltd</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>EIT Health application portal</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Up to EUR 850,000, max 50% co-funding</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Sami + Valerio</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Missing research/education partner and IML6 evidence pack</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Treat as next-wave target after partner and maturity evidence are assembled</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>GRANT_APPLICATIONS_STATUS.md</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Open call with real fit, but not immediate from current repo assets</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>